<commit_message>
EPBDS-16836 Fix min dropping NaN while max returned it, because both ranked NaN above every number, so min(NaN, 1.5) was 1.5
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Numbers.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Numbers.xlsx
@@ -5889,7 +5889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I41"/>
+  <dimension ref="B2:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -5908,7 +5908,7 @@
     <row r="4" ht="43.5" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>isNaN and isInfinite check Double and Float values; an empty value is neither. isInfinite also treats the limits of Integer and Long, MIN_VALUE and MAX_VALUE, as infinite. isEmpty is true only for an empty value, not for 0. NaN is not equal to anything, and "&lt;" or "&gt;" with NaN gives an empty result. toString writes infinity as the sign "∞".</t>
+          <t>isNaN and isInfinite check Double and Float values; an empty value is neither. isInfinite also treats the limits of Integer and Long, MIN_VALUE and MAX_VALUE, as infinite. isEmpty is true only for an empty value, not for 0. NaN is not equal to anything, and "&lt;" or "&gt;" with NaN gives an empty result, while min and max with NaN give NaN, whatever the order of the arguments. toString writes infinity as the sign "∞".</t>
         </is>
       </c>
     </row>
@@ -5959,253 +5959,238 @@
     <row r="10">
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>InfinityGreater</t>
+          <t>NaNMax</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>= 1.0 / 0 &gt; Double.MAX_VALUE</t>
+          <t>= max(Double.NaN, 1.5)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>EmptyIsNaN</t>
+          <t>NaNMin</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>= Double v = null; isNaN(v)</t>
+          <t>= min(1.5, Double.NaN)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>EmptyIsInfinite</t>
+          <t>FloatNaNMin</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>= Double v = null; isInfinite(v)</t>
+          <t>= min(new float[] {Float.NaN, 1.5f})</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>EmptyIsEmpty</t>
+          <t>InfinityGreater</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>= Double v = null; isEmpty(v)</t>
+          <t>= 1.0 / 0 &gt; Double.MAX_VALUE</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>ZeroIsEmpty</t>
+          <t>EmptyIsNaN</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>= isEmpty(0.0)</t>
+          <t>= Double v = null; isNaN(v)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>FloatNaN</t>
+          <t>EmptyIsInfinite</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>= isNaN(Float.NaN)</t>
+          <t>= Double v = null; isInfinite(v)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>FloatInfinite</t>
+          <t>EmptyIsEmpty</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>= isInfinite(Float.NEGATIVE_INFINITY)</t>
+          <t>= Double v = null; isEmpty(v)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>LongLimitInfinite</t>
+          <t>ZeroIsEmpty</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>= isInfinite(Long.MAX_VALUE)</t>
+          <t>= isEmpty(0.0)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>IntegerLimitInfinite</t>
+          <t>FloatNaN</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>= isInfinite(Integer.MIN_VALUE)</t>
+          <t>= isNaN(Float.NaN)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>NearLimitFinite</t>
+          <t>FloatInfinite</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>= isInfinite(Long.MAX_VALUE - 1)</t>
+          <t>= isInfinite(Float.NEGATIVE_INFINITY)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>WholeIsNaN</t>
+          <t>LongLimitInfinite</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>= isNaN(5L)</t>
+          <t>= isInfinite(Long.MAX_VALUE)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>InfinityText</t>
+          <t>IntegerLimitInfinite</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>= toString(1.0 / 0)</t>
+          <t>= isInfinite(Integer.MIN_VALUE)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>NegativeInfinityText</t>
+          <t>NearLimitFinite</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>= toString(-1.0 / 0)</t>
+          <t>= isInfinite(Long.MAX_VALUE - 1)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="6" t="inlineStr">
         <is>
+          <t>WholeIsNaN</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>= isNaN(5L)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>InfinityText</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>= toString(1.0 / 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>NegativeInfinityText</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>= toString(-1.0 / 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="6" t="inlineStr">
+        <is>
           <t>NaNText</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>= toString(0.0 / 0)</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Test SpecialValueChecks SpecialValueChecksTest</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="4" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$NaNGreater</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Double v = Double.NaN; v &gt; 0</t>
-        </is>
-      </c>
-      <c r="D26" s="10" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$NaNEqualsZero</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Double v = Double.NaN; v == 0</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$InfinityGreater</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>1.0 / 0 &gt; Double.MAX_VALUE</t>
-        </is>
-      </c>
-      <c r="D28" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyIsNaN</t>
+          <t>_res_.$NaNGreater</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; isNaN(v)</t>
-        </is>
-      </c>
-      <c r="D29" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
+          <t>Double v = Double.NaN; v &gt; 0</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyIsInfinite</t>
+          <t>_res_.$NaNEqualsZero</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; isInfinite(v)</t>
+          <t>Double v = Double.NaN; v == 0</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
@@ -6217,63 +6202,63 @@
     <row r="31">
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyIsEmpty</t>
+          <t>_res_.$NaNMax</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Double v = null; isEmpty(v)</t>
+          <t>max(Double.NaN, 1.5)</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>NaN</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ZeroIsEmpty</t>
+          <t>_res_.$NaNMin</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>isEmpty(0.0)</t>
+          <t>min(1.5, Double.NaN)</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>NaN</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>_res_.$FloatNaN</t>
+          <t>_res_.$FloatNaNMin</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>isNaN(Float.NaN)</t>
+          <t>min(new float[] {Float.NaN, 1.5f})</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>NaN</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>_res_.$FloatInfinite</t>
+          <t>_res_.$InfinityGreater</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>isInfinite(Float.NEGATIVE_INFINITY)</t>
+          <t>1.0 / 0 &gt; Double.MAX_VALUE</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
@@ -6285,63 +6270,63 @@
     <row r="35">
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>_res_.$LongLimitInfinite</t>
+          <t>_res_.$EmptyIsNaN</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>isInfinite(Long.MAX_VALUE)</t>
+          <t>Double v = null; isNaN(v)</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="9" t="inlineStr">
         <is>
-          <t>_res_.$IntegerLimitInfinite</t>
+          <t>_res_.$EmptyIsInfinite</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>isInfinite(Integer.MIN_VALUE)</t>
+          <t>Double v = null; isInfinite(v)</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NearLimitFinite</t>
+          <t>_res_.$EmptyIsEmpty</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>isInfinite(Long.MAX_VALUE - 1)</t>
+          <t>Double v = null; isEmpty(v)</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="9" t="inlineStr">
         <is>
-          <t>_res_.$WholeIsNaN</t>
+          <t>_res_.$ZeroIsEmpty</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>isNaN(5L)</t>
+          <t>isEmpty(0.0)</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
@@ -6353,49 +6338,151 @@
     <row r="39">
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>_res_.$InfinityText</t>
+          <t>_res_.$FloatNaN</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>toString(1.0 / 0)</t>
+          <t>isNaN(Float.NaN)</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>∞</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NegativeInfinityText</t>
+          <t>_res_.$FloatInfinite</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>toString(-1.0 / 0)</t>
+          <t>isInfinite(Float.NEGATIVE_INFINITY)</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>-∞</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="9" t="inlineStr">
         <is>
+          <t>_res_.$LongLimitInfinite</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>isInfinite(Long.MAX_VALUE)</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$IntegerLimitInfinite</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>isInfinite(Integer.MIN_VALUE)</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NearLimitFinite</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>isInfinite(Long.MAX_VALUE - 1)</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$WholeIsNaN</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>isNaN(5L)</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$InfinityText</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>toString(1.0 / 0)</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>∞</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NegativeInfinityText</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>toString(-1.0 / 0)</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>-∞</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="9" t="inlineStr">
+        <is>
           <t>_res_.$NaNText</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>toString(0.0 / 0)</t>
         </is>
       </c>
-      <c r="D41" s="10" t="inlineStr">
+      <c r="D47" s="10" t="inlineStr">
         <is>
           <t>NaN</t>
         </is>
@@ -6404,7 +6491,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
EPBDS-16840 Fix math functions reading an empty argument as 0, so cos(v) was 1
Add abs of BigDecimal and BigInteger, which did not compile.
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Numbers.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Numbers.xlsx
@@ -1431,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I60"/>
+  <dimension ref="B2:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1758,10 +1758,10 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1">
+    <row r="33" ht="30" customHeight="1">
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>pow(null, 2) counts the empty base as 0. A Double keeps about 16 digits, so a big exact power is computed with the pow method of BigInteger.</t>
+          <t>pow of an empty base or an empty exponent is empty, as every math function of an empty argument is. A Double keeps about 16 digits, so a big exact power is computed with the pow method of BigInteger.</t>
         </is>
       </c>
     </row>
@@ -1896,206 +1896,229 @@
     <row r="46">
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>BeyondDoublePrecision</t>
+          <t>EmptyExponent</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
         <is>
-          <t>= (Long) pow(2, 62)</t>
+          <t>= pow(2, null)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" s="6" t="inlineStr">
         <is>
+          <t>BeyondDoublePrecision</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>= (Long) pow(2, 62)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="6" t="inlineStr">
+        <is>
           <t>ExactBigPower</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C48" s="7" t="inlineStr">
         <is>
           <t>= new BigInteger("2").pow(100)</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" s="3" t="inlineStr">
+    <row r="50">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Test PowerEdgeCases PowerEdgeCasesTest</t>
         </is>
       </c>
-      <c r="C49" s="8" t="n"/>
-      <c r="D49" s="4" t="n"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$WholePower</t>
-        </is>
-      </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>pow(2, 10)</t>
-        </is>
-      </c>
-      <c r="D50" s="10" t="n">
-        <v>1024</v>
-      </c>
+      <c r="C50" s="8" t="n"/>
+      <c r="D50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="B51" s="9" t="inlineStr">
         <is>
-          <t>_res_.$PowerType</t>
+          <t>_res_.$WholePower</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>((Double) pow(2, 10)).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D51" s="10" t="inlineStr">
-        <is>
-          <t>Double</t>
-        </is>
+          <t>pow(2, 10)</t>
+        </is>
+      </c>
+      <c r="D51" s="10" t="n">
+        <v>1024</v>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NegativeExponent</t>
+          <t>_res_.$PowerType</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>pow(2, -1)</t>
-        </is>
-      </c>
-      <c r="D52" s="10" t="n">
-        <v>0.5</v>
+          <t>((Double) pow(2, 10)).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ZeroToZero</t>
+          <t>_res_.$NegativeExponent</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>pow(0, 0)</t>
+          <t>pow(2, -1)</t>
         </is>
       </c>
       <c r="D53" s="10" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>_res_.$SquareRoot</t>
+          <t>_res_.$ZeroToZero</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>pow(2, 0.5)</t>
+          <t>pow(0, 0)</t>
         </is>
       </c>
       <c r="D54" s="10" t="n">
-        <v>1.414213562373095</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NegativeBase</t>
+          <t>_res_.$SquareRoot</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>pow(-2, 3)</t>
+          <t>pow(2, 0.5)</t>
         </is>
       </c>
       <c r="D55" s="10" t="n">
-        <v>-8</v>
+        <v>1.414213562373095</v>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RootOfNegative</t>
+          <t>_res_.$NegativeBase</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>isNaN(pow(-8, 1.0 / 3))</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>pow(-2, 3)</t>
+        </is>
+      </c>
+      <c r="D56" s="10" t="n">
+        <v>-8</v>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>_res_.$TooBig</t>
+          <t>_res_.$RootOfNegative</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>pow(10, 309)</t>
+          <t>isNaN(pow(-8, 1.0 / 3))</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>Infinity</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyBase</t>
+          <t>_res_.$TooBig</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>pow(null, 2)</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="n">
-        <v>0</v>
+          <t>pow(10, 309)</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>Infinity</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BeyondDoublePrecision</t>
+          <t>_res_.$EmptyBase</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>(Long) pow(2, 62)</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="inlineStr">
-        <is>
-          <t>4611686018427387904</t>
-        </is>
-      </c>
+          <t>pow(null, 2)</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="n"/>
     </row>
     <row r="60">
       <c r="B60" s="9" t="inlineStr">
         <is>
+          <t>_res_.$EmptyExponent</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>pow(2, null)</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="n"/>
+    </row>
+    <row r="61">
+      <c r="B61" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$BeyondDoublePrecision</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>(Long) pow(2, 62)</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="inlineStr">
+        <is>
+          <t>4611686018427387904</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="9" t="inlineStr">
+        <is>
           <t>_res_.$ExactBigPower</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr">
         <is>
           <t>new BigInteger("2").pow(100)</t>
         </is>
       </c>
-      <c r="D60" s="10" t="inlineStr">
+      <c r="D62" s="10" t="inlineStr">
         <is>
           <t>1267650600228229401496703205376</t>
         </is>
@@ -2105,7 +2128,7 @@
   <mergeCells count="7">
     <mergeCell ref="B33:I33"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B50:D50"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B35:C35"/>
@@ -4579,10 +4602,10 @@
         <v>195</v>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1">
+    <row r="51" ht="30" customHeight="1">
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>An empty operand counts as 0 for "+" and "-" and makes "*" and "/" empty, for every number type. Negating an empty value gives an empty value.</t>
+          <t>An empty operand counts as 0 for "+" and "-" and makes "*" and "/" empty, for every number type. Negating an empty value gives an empty value, and so does a math function of an empty argument, as the EmptyValues sheet shows.</t>
         </is>
       </c>
     </row>
@@ -4865,7 +4888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I87"/>
+  <dimension ref="B2:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -4874,6 +4897,8 @@
     <col width="24.1" customWidth="1" min="4" max="4"/>
     <col width="16.7" customWidth="1" min="5" max="5"/>
     <col width="13.6" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="21.9" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -5719,10 +5744,10 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="16.5" customHeight="1">
+    <row r="74" ht="30" customHeight="1">
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>A spreadsheet step with a type and no formula holds the default value of the type: 0 and false for the primitive types int, double and boolean, empty for Integer, String and the other object types.</t>
+          <t>A spreadsheet step with a type and no formula holds the default value of the type: 0 and false for the primitive types int, double and boolean, empty for Integer, String and the other object types. A math function follows that value: abs of the double step is 0, abs of the Integer step is empty.</t>
         </is>
       </c>
     </row>
@@ -5786,85 +5811,135 @@
       </c>
       <c r="C82" s="6" t="n"/>
     </row>
+    <row r="83">
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>AbsOfFraction</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>= abs($Fraction)</t>
+        </is>
+      </c>
+    </row>
     <row r="84">
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>AbsOfWrapper</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>= abs($Wrapper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>Test EmptyTypedSteps EmptyTypedStepsTest</t>
         </is>
       </c>
-      <c r="C84" s="8" t="n"/>
-      <c r="D84" s="8" t="n"/>
-      <c r="E84" s="8" t="n"/>
-      <c r="F84" s="4" t="n"/>
-    </row>
-    <row r="85">
-      <c r="B85" s="9" t="inlineStr">
+      <c r="C86" s="8" t="n"/>
+      <c r="D86" s="8" t="n"/>
+      <c r="E86" s="8" t="n"/>
+      <c r="F86" s="8" t="n"/>
+      <c r="G86" s="8" t="n"/>
+      <c r="H86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="9" t="inlineStr">
         <is>
           <t>_res_.$WholeNumber</t>
         </is>
       </c>
-      <c r="C85" s="9" t="inlineStr">
+      <c r="C87" s="9" t="inlineStr">
         <is>
           <t>_res_.$Fraction</t>
         </is>
       </c>
-      <c r="D85" s="9" t="inlineStr">
+      <c r="D87" s="9" t="inlineStr">
         <is>
           <t>_res_.$Flag</t>
         </is>
       </c>
-      <c r="E85" s="9" t="inlineStr">
+      <c r="E87" s="9" t="inlineStr">
         <is>
           <t>_res_.$Wrapper</t>
         </is>
       </c>
-      <c r="F85" s="9" t="inlineStr">
+      <c r="F87" s="9" t="inlineStr">
         <is>
           <t>_res_.$Text</t>
         </is>
       </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="5" t="inlineStr">
+      <c r="G87" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$AbsOfFraction</t>
+        </is>
+      </c>
+      <c r="H87" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$AbsOfWrapper</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="5" t="inlineStr">
         <is>
           <t>int</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr">
+      <c r="C88" s="5" t="inlineStr">
         <is>
           <t>double</t>
         </is>
       </c>
-      <c r="D86" s="5" t="inlineStr">
+      <c r="D88" s="5" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="E86" s="5" t="inlineStr">
+      <c r="E88" s="5" t="inlineStr">
         <is>
           <t>Integer</t>
         </is>
       </c>
-      <c r="F86" s="5" t="inlineStr">
+      <c r="F88" s="5" t="inlineStr">
         <is>
           <t>String</t>
         </is>
       </c>
-    </row>
-    <row r="87">
-      <c r="B87" s="10" t="n">
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>abs($Fraction)</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>abs($Wrapper)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="C87" s="10" t="n">
+      <c r="C89" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="D87" s="10" t="inlineStr">
+      <c r="D89" s="10" t="inlineStr">
         <is>
           <t>false</t>
         </is>
       </c>
-      <c r="E87" s="10" t="n"/>
-      <c r="F87" s="10" t="n"/>
+      <c r="E89" s="10" t="n"/>
+      <c r="F89" s="10" t="n"/>
+      <c r="G89" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -5875,7 +5950,7 @@
     <mergeCell ref="B76:C76"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B65:D65"/>
-    <mergeCell ref="B84:F84"/>
+    <mergeCell ref="B86:H86"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6505,11 +6580,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:J49"/>
+  <dimension ref="B2:J127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="17.8" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
     <col width="70" customWidth="1" min="3" max="3"/>
     <col width="15.7" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
@@ -6523,7 +6598,7 @@
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Empty values in logic and in objects</t>
+          <t>Empty values in logic, in objects and in math functions</t>
         </is>
       </c>
     </row>
@@ -7257,8 +7332,939 @@
       <c r="F49" s="10" t="n"/>
       <c r="G49" s="10" t="n"/>
     </row>
+    <row r="51" ht="16.5" customHeight="1">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Every math function returns an empty value when an argument is empty, unlike "+" and "-", which count an empty operand as 0. isNaN and isInfinite check a value, so they are false for an empty one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Spreadsheet SpreadsheetResult EmptyMathArguments()</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="n"/>
+    </row>
+    <row r="54">
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>Empty</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>= (Double) null</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>= abs($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>AbsOfDecimal</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>= abs((BigDecimal) null)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>Acos</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>= acos($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>Asin</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>= asin($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>Atan</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>= atan($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>Cbrt</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>= cbrt($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Ceil</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>= ceil($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Cos</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>= cos($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>Cosh</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>= cosh($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>Exp</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>= exp($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>Expm1</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>= expm1($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>= floor($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>Exponent</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>= getExponent($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>Log</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>= log($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>Log10</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>= log10($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Log1p</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>= log1p($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>NextUp</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>= nextAfter($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>Rint</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>= rint($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>Signum</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>= signum($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>Sin</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>= sin($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Sinh</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>= sinh($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Sqrt</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>= sqrt($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>Tan</t>
+        </is>
+      </c>
+      <c r="C78" s="7" t="inlineStr">
+        <is>
+          <t>= tan($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>Tanh</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>= tanh($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>ToDegrees</t>
+        </is>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
+          <t>= toDegrees($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>ToRadians</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>= toRadians($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>Ulp</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>= ulp($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>Atan2</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>= atan2($Empty, 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>CopySign</t>
+        </is>
+      </c>
+      <c r="C84" s="7" t="inlineStr">
+        <is>
+          <t>= copySign(1.0, $Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>Hypotenuse</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>= getExponent(3, $Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>IeeeRemainder</t>
+        </is>
+      </c>
+      <c r="C86" s="7" t="inlineStr">
+        <is>
+          <t>= IEEEremainder($Empty, 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>NextAfter</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>= nextAfter(1.0, $Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>Scalb</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr">
+        <is>
+          <t>= scalb($Empty, 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>IsNaN</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>= isNaN($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>IsInfinite</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr">
+        <is>
+          <t>= isInfinite($Empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Test EmptyMathArguments EmptyMathArgumentsTest</t>
+        </is>
+      </c>
+      <c r="C92" s="8" t="n"/>
+      <c r="D92" s="4" t="n"/>
+    </row>
+    <row r="93">
+      <c r="B93" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Abs</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>abs($Empty)</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="n"/>
+    </row>
+    <row r="94">
+      <c r="B94" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$AbsOfDecimal</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>abs((BigDecimal) null)</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="n"/>
+    </row>
+    <row r="95">
+      <c r="B95" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Acos</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>acos($Empty)</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="n"/>
+    </row>
+    <row r="96">
+      <c r="B96" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Asin</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>asin($Empty)</t>
+        </is>
+      </c>
+      <c r="D96" s="10" t="n"/>
+    </row>
+    <row r="97">
+      <c r="B97" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Atan</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>atan($Empty)</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="n"/>
+    </row>
+    <row r="98">
+      <c r="B98" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Cbrt</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr">
+        <is>
+          <t>cbrt($Empty)</t>
+        </is>
+      </c>
+      <c r="D98" s="10" t="n"/>
+    </row>
+    <row r="99">
+      <c r="B99" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Ceil</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>ceil($Empty)</t>
+        </is>
+      </c>
+      <c r="D99" s="10" t="n"/>
+    </row>
+    <row r="100">
+      <c r="B100" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Cos</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>cos($Empty)</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="n"/>
+    </row>
+    <row r="101">
+      <c r="B101" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Cosh</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>cosh($Empty)</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="n"/>
+    </row>
+    <row r="102">
+      <c r="B102" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Exp</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>exp($Empty)</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="n"/>
+    </row>
+    <row r="103">
+      <c r="B103" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Expm1</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>expm1($Empty)</t>
+        </is>
+      </c>
+      <c r="D103" s="10" t="n"/>
+    </row>
+    <row r="104">
+      <c r="B104" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Floor</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>floor($Empty)</t>
+        </is>
+      </c>
+      <c r="D104" s="10" t="n"/>
+    </row>
+    <row r="105">
+      <c r="B105" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Exponent</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>getExponent($Empty)</t>
+        </is>
+      </c>
+      <c r="D105" s="10" t="n"/>
+    </row>
+    <row r="106">
+      <c r="B106" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Log</t>
+        </is>
+      </c>
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>log($Empty)</t>
+        </is>
+      </c>
+      <c r="D106" s="10" t="n"/>
+    </row>
+    <row r="107">
+      <c r="B107" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Log10</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>log10($Empty)</t>
+        </is>
+      </c>
+      <c r="D107" s="10" t="n"/>
+    </row>
+    <row r="108">
+      <c r="B108" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Log1p</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>log1p($Empty)</t>
+        </is>
+      </c>
+      <c r="D108" s="10" t="n"/>
+    </row>
+    <row r="109">
+      <c r="B109" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NextUp</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>nextAfter($Empty)</t>
+        </is>
+      </c>
+      <c r="D109" s="10" t="n"/>
+    </row>
+    <row r="110">
+      <c r="B110" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Rint</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>rint($Empty)</t>
+        </is>
+      </c>
+      <c r="D110" s="10" t="n"/>
+    </row>
+    <row r="111">
+      <c r="B111" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Signum</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>signum($Empty)</t>
+        </is>
+      </c>
+      <c r="D111" s="10" t="n"/>
+    </row>
+    <row r="112">
+      <c r="B112" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Sin</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>sin($Empty)</t>
+        </is>
+      </c>
+      <c r="D112" s="10" t="n"/>
+    </row>
+    <row r="113">
+      <c r="B113" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Sinh</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>sinh($Empty)</t>
+        </is>
+      </c>
+      <c r="D113" s="10" t="n"/>
+    </row>
+    <row r="114">
+      <c r="B114" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Sqrt</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>sqrt($Empty)</t>
+        </is>
+      </c>
+      <c r="D114" s="10" t="n"/>
+    </row>
+    <row r="115">
+      <c r="B115" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Tan</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>tan($Empty)</t>
+        </is>
+      </c>
+      <c r="D115" s="10" t="n"/>
+    </row>
+    <row r="116">
+      <c r="B116" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Tanh</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>tanh($Empty)</t>
+        </is>
+      </c>
+      <c r="D116" s="10" t="n"/>
+    </row>
+    <row r="117">
+      <c r="B117" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ToDegrees</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>toDegrees($Empty)</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="n"/>
+    </row>
+    <row r="118">
+      <c r="B118" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$ToRadians</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>toRadians($Empty)</t>
+        </is>
+      </c>
+      <c r="D118" s="10" t="n"/>
+    </row>
+    <row r="119">
+      <c r="B119" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Ulp</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>ulp($Empty)</t>
+        </is>
+      </c>
+      <c r="D119" s="10" t="n"/>
+    </row>
+    <row r="120">
+      <c r="B120" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Atan2</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>atan2($Empty, 1)</t>
+        </is>
+      </c>
+      <c r="D120" s="10" t="n"/>
+    </row>
+    <row r="121">
+      <c r="B121" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$CopySign</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>copySign(1.0, $Empty)</t>
+        </is>
+      </c>
+      <c r="D121" s="10" t="n"/>
+    </row>
+    <row r="122">
+      <c r="B122" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Hypotenuse</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>getExponent(3, $Empty)</t>
+        </is>
+      </c>
+      <c r="D122" s="10" t="n"/>
+    </row>
+    <row r="123">
+      <c r="B123" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$IeeeRemainder</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>IEEEremainder($Empty, 3)</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="n"/>
+    </row>
+    <row r="124">
+      <c r="B124" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$NextAfter</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>nextAfter(1.0, $Empty)</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="n"/>
+    </row>
+    <row r="125">
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$Scalb</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>scalb($Empty, 3)</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="n"/>
+    </row>
+    <row r="126">
+      <c r="B126" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$IsNaN</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>isNaN($Empty)</t>
+        </is>
+      </c>
+      <c r="D126" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$IsInfinite</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>isInfinite($Empty)</t>
+        </is>
+      </c>
+      <c r="D127" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="11">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B46:G46"/>
     <mergeCell ref="B25:I25"/>
@@ -7267,6 +8273,9 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="B16:J16"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B92:D92"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
EPBDS-9967 Restore % and ** as aliases of remainder and pow, add exact big pow
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Numbers.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Numbers.xlsx
@@ -1039,10 +1039,10 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B6:I6"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B6:I6"/>
     <mergeCell ref="B4:I4"/>
-    <mergeCell ref="B26:D26"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -1415,8 +1415,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B6:I6"/>
     <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B6:I6"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
@@ -1431,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I62"/>
+  <dimension ref="B2:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1450,7 +1450,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Formulas have no "%" and "**" operators: remainder(x, y) returns the remainder with the sign of x, as "%" in Java does, and pow(x, y) raises x to the power y. "10%" is a percent literal, 0.1. remainder keeps the type of its operands; pow always returns a Double.</t>
+          <t>remainder(x, y) returns the remainder with the sign of x, as "%" in Java does, and pow(x, y) raises x to the power y. x % y and x ** y are their short forms, shown in the Operators workbook. "10%" is a percent literal, 0.1. remainder keeps the type of its operands; pow returns a Double, except for a BigInteger or a BigDecimal raised to a whole power.</t>
         </is>
       </c>
     </row>
@@ -1761,7 +1761,7 @@
     <row r="33" ht="30" customHeight="1">
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>pow of an empty base or an empty exponent is empty, as every math function of an empty argument is. A Double keeps about 16 digits, so a big exact power is computed with the pow method of BigInteger.</t>
+          <t>pow of an empty base or an empty exponent is empty, as every math function of an empty argument is. A Double keeps about 16 digits, so for a big exact power pass a BigInteger or a BigDecimal and a whole exponent. With a negative exponent a BigDecimal power is 1 divided by the power, rounded to 34 digits.</t>
         </is>
       </c>
     </row>
@@ -1925,167 +1925,166 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>= new BigInteger("2").pow(100)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="B50" s="3" t="inlineStr">
+          <t>= pow(new BigInteger("2"), 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>DecimalInversePower</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>= pow(new BigDecimal("3"), -1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>Test PowerEdgeCases PowerEdgeCasesTest</t>
         </is>
       </c>
-      <c r="C50" s="8" t="n"/>
-      <c r="D50" s="4" t="n"/>
-    </row>
-    <row r="51">
-      <c r="B51" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$WholePower</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>pow(2, 10)</t>
-        </is>
-      </c>
-      <c r="D51" s="10" t="n">
-        <v>1024</v>
-      </c>
+      <c r="C51" s="8" t="n"/>
+      <c r="D51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>_res_.$PowerType</t>
+          <t>_res_.$WholePower</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>((Double) pow(2, 10)).getClass().getSimpleName()</t>
-        </is>
-      </c>
-      <c r="D52" s="10" t="inlineStr">
-        <is>
-          <t>Double</t>
-        </is>
+          <t>pow(2, 10)</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="n">
+        <v>1024</v>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NegativeExponent</t>
+          <t>_res_.$PowerType</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>pow(2, -1)</t>
-        </is>
-      </c>
-      <c r="D53" s="10" t="n">
-        <v>0.5</v>
+          <t>((Double) pow(2, 10)).getClass().getSimpleName()</t>
+        </is>
+      </c>
+      <c r="D53" s="10" t="inlineStr">
+        <is>
+          <t>Double</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>_res_.$ZeroToZero</t>
+          <t>_res_.$NegativeExponent</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>pow(0, 0)</t>
+          <t>pow(2, -1)</t>
         </is>
       </c>
       <c r="D54" s="10" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="9" t="inlineStr">
         <is>
-          <t>_res_.$SquareRoot</t>
+          <t>_res_.$ZeroToZero</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>pow(2, 0.5)</t>
+          <t>pow(0, 0)</t>
         </is>
       </c>
       <c r="D55" s="10" t="n">
-        <v>1.414213562373095</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="9" t="inlineStr">
         <is>
-          <t>_res_.$NegativeBase</t>
+          <t>_res_.$SquareRoot</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>pow(-2, 3)</t>
+          <t>pow(2, 0.5)</t>
         </is>
       </c>
       <c r="D56" s="10" t="n">
-        <v>-8</v>
+        <v>1.414213562373095</v>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="9" t="inlineStr">
         <is>
-          <t>_res_.$RootOfNegative</t>
+          <t>_res_.$NegativeBase</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>isNaN(pow(-8, 1.0 / 3))</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t>pow(-2, 3)</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="n">
+        <v>-8</v>
       </c>
     </row>
     <row r="58">
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>_res_.$TooBig</t>
+          <t>_res_.$RootOfNegative</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>pow(10, 309)</t>
+          <t>isNaN(pow(-8, 1.0 / 3))</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>Infinity</t>
+          <t>true</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyBase</t>
+          <t>_res_.$TooBig</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>pow(null, 2)</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="n"/>
+          <t>pow(10, 309)</t>
+        </is>
+      </c>
+      <c r="D59" s="10" t="inlineStr">
+        <is>
+          <t>Infinity</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>_res_.$EmptyExponent</t>
+          <t>_res_.$EmptyBase</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>pow(2, null)</t>
+          <t>pow(null, 2)</t>
         </is>
       </c>
       <c r="D60" s="10" t="n"/>
@@ -2093,34 +2092,64 @@
     <row r="61">
       <c r="B61" s="9" t="inlineStr">
         <is>
-          <t>_res_.$BeyondDoublePrecision</t>
+          <t>_res_.$EmptyExponent</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>(Long) pow(2, 62)</t>
-        </is>
-      </c>
-      <c r="D61" s="10" t="inlineStr">
-        <is>
-          <t>4611686018427387904</t>
-        </is>
-      </c>
+          <t>pow(2, null)</t>
+        </is>
+      </c>
+      <c r="D61" s="10" t="n"/>
     </row>
     <row r="62">
       <c r="B62" s="9" t="inlineStr">
         <is>
+          <t>_res_.$BeyondDoublePrecision</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>(Long) pow(2, 62)</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>4611686018427387904</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="B63" s="9" t="inlineStr">
+        <is>
           <t>_res_.$ExactBigPower</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>new BigInteger("2").pow(100)</t>
-        </is>
-      </c>
-      <c r="D62" s="10" t="inlineStr">
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>pow(new BigInteger("2"), 100)</t>
+        </is>
+      </c>
+      <c r="D63" s="10" t="inlineStr">
         <is>
           <t>1267650600228229401496703205376</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="9" t="inlineStr">
+        <is>
+          <t>_res_.$DecimalInversePower</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>pow(new BigDecimal("3"), -1)</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>0.3333333333333333333333333333333333</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2157,7 @@
   <mergeCells count="7">
     <mergeCell ref="B33:I33"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="B51:D51"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B35:C35"/>
@@ -5943,14 +5972,14 @@
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B74:I74"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="B55:C55"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B74:I74"/>
     <mergeCell ref="B53:I53"/>
     <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B86:H86"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B65:D65"/>
-    <mergeCell ref="B86:H86"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6565,8 +6594,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B28:D28"/>
     <mergeCell ref="B4:I4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8268,14 +8297,14 @@
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B46:G46"/>
     <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B51:I51"/>
     <mergeCell ref="B41:J41"/>
+    <mergeCell ref="B92:D92"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B53:C53"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="B16:J16"/>
-    <mergeCell ref="B51:I51"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B92:D92"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
EPBDS-7362 Compute Double arithmetic with the decimals the numbers show
The binary rounding of + - * / % ++ -- on Double was reported in:

- EPBDS-7362 0.1 + 0.05 - 0.03 is 0.12000000000000002
- EPBDS-7841 (1 - 0.9) * 1042.35 rounds to 104.23, not 104.24
- EPBDS-3786 0.7 * 0.75 rounds to 0.52, not 0.53
- EPBDS-5243 a calculation gives 268.59000000000003, not 268.59
- EPBDS-9106 a test shows 268.59000000000003, not 268.59
- EPBDS-7893 a test of 40.0499999999999 * 1.03 fails though it looks equal
- EPBDS-13543 a test fails on 0.08334 but passes on 20.76
- EPBDS-16890 a test shows 1.73 * 12 as 20.759999999999998
- EPBDS-16891 a run shows 1.73 * 12 as 20.759999999999998
- EPBDS-17023 (Double)16.85 * 100 % 2 is 1.0000000000002274
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Numbers.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/6-Language/Numbers.xlsx
@@ -17,9 +17,25 @@
     <sheet name="SpecialValues" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="EmptyValues" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+  <si>
+    <t>Byte, Short, Integer and Long arithmetic wraps around past the limit without an error, so cast an operand to a wider type first. A cast to a whole type drops the fraction toward zero, keeps only the low bits of a too big whole number, and saturates a too big fraction at the limit. Double division by zero gives Infinity, and 0.0 / 0.0 gives NaN. Double arithmetic computes with the decimals the numbers show, as a calculator does, so 0.1 + 0.2 is exactly 0.3.</t>
+  </si>
+  <si>
+    <t>DecimalFraction</t>
+  </si>
+  <si>
+    <t>_res_.$DecimalFraction</t>
+  </si>
+  <si>
+    <t>true</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -555,13 +571,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I41"/>
+  <dimension ref="B2:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="21.9" customWidth="1" min="2" max="2"/>
-    <col width="58.7" customWidth="1" min="3" max="3"/>
-    <col width="39.8" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="21.9"/>
+    <col min="3" max="3" customWidth="true" width="58.7"/>
+    <col min="4" max="4" customWidth="true" width="39.8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1055,13 +1071,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I33"/>
+  <dimension ref="B2:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="30.4" customWidth="1" min="2" max="2"/>
-    <col width="55.6" customWidth="1" min="3" max="3"/>
-    <col width="12.5" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="30.4"/>
+    <col min="3" max="3" customWidth="true" width="55.6"/>
+    <col min="4" max="4" customWidth="true" width="12.5"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1431,13 +1447,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I64"/>
+  <dimension ref="B2:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="31.4" customWidth="1" min="2" max="2"/>
-    <col width="54.5" customWidth="1" min="3" max="3"/>
-    <col width="34.6" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="31.4"/>
+    <col min="3" max="3" customWidth="true" width="54.5"/>
+    <col min="4" max="4" customWidth="true" width="34.6"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2174,13 +2190,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I45"/>
+  <dimension ref="B2:D45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="29.3" customWidth="1" min="2" max="2"/>
-    <col width="64" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="29.3"/>
+    <col min="3" max="3" customWidth="true" width="64.0"/>
+    <col min="4" max="4" customWidth="true" width="23.0"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -2191,10 +2207,8 @@
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Byte, Short, Integer and Long arithmetic wraps around past the limit without an error, so cast an operand to a wider type first. A cast to a whole type drops the fraction toward zero, keeps only the low bits of a too big whole number, and saturates a too big fraction at the limit. Double division by zero gives Infinity, and 0.0 / 0.0 gives NaN.</t>
-        </is>
+      <c r="B4" s="2" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -2410,10 +2424,8 @@
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>BinaryFraction</t>
-        </is>
+      <c r="B24" s="6" t="s">
+        <v>1</v>
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
@@ -2699,20 +2711,16 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="9" t="inlineStr">
-        <is>
-          <t>_res_.$BinaryFraction</t>
-        </is>
+      <c r="B44" s="9" t="s">
+        <v>2</v>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
           <t>0.1 + 0.2 ==== 0.3</t>
         </is>
       </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="D44" s="10" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="45">
@@ -2752,17 +2760,17 @@
   <dimension ref="B2:K92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="33.9" customWidth="1" min="2" max="2"/>
-    <col width="52.4" customWidth="1" min="3" max="3"/>
-    <col width="19.9" customWidth="1" min="4" max="4"/>
-    <col width="21.9" customWidth="1" min="5" max="5"/>
-    <col width="21.9" customWidth="1" min="6" max="6"/>
-    <col width="19.9" customWidth="1" min="7" max="7"/>
-    <col width="20.9" customWidth="1" min="8" max="8"/>
-    <col width="33.5" customWidth="1" min="9" max="9"/>
-    <col width="25.1" customWidth="1" min="10" max="10"/>
-    <col width="21.9" customWidth="1" min="11" max="11"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="33.9"/>
+    <col min="3" max="3" customWidth="true" width="52.4"/>
+    <col min="4" max="4" customWidth="true" width="19.9"/>
+    <col min="5" max="5" customWidth="true" width="21.9"/>
+    <col min="6" max="6" customWidth="true" width="21.9"/>
+    <col min="7" max="7" customWidth="true" width="19.9"/>
+    <col min="8" max="8" customWidth="true" width="20.9"/>
+    <col min="9" max="9" customWidth="true" width="33.5"/>
+    <col min="10" max="10" customWidth="true" width="25.1"/>
+    <col min="11" max="11" customWidth="true" width="21.9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -4047,13 +4055,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I74"/>
+  <dimension ref="B2:D74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="35.6" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="39.8" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="35.6"/>
+    <col min="3" max="3" customWidth="true" width="70.0"/>
+    <col min="4" max="4" customWidth="true" width="39.8"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -4917,17 +4925,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I89"/>
+  <dimension ref="B2:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="32.5" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="24.1" customWidth="1" min="4" max="4"/>
-    <col width="16.7" customWidth="1" min="5" max="5"/>
-    <col width="13.6" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="21.9" customWidth="1" min="8" max="8"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="32.5"/>
+    <col min="3" max="3" customWidth="true" width="70.0"/>
+    <col min="4" max="4" customWidth="true" width="24.1"/>
+    <col min="5" max="5" customWidth="true" width="16.7"/>
+    <col min="6" max="6" customWidth="true" width="13.6"/>
+    <col min="7" max="7" customWidth="true" width="23.0"/>
+    <col min="8" max="8" customWidth="true" width="21.9"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -5993,13 +6001,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I47"/>
+  <dimension ref="B2:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="30.4" customWidth="1" min="2" max="2"/>
-    <col width="40.9" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="30.4"/>
+    <col min="3" max="3" customWidth="true" width="40.9"/>
+    <col min="4" max="4" customWidth="true" width="10.0"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -6612,16 +6620,16 @@
   <dimension ref="B2:J127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="70" customWidth="1" min="3" max="3"/>
-    <col width="15.7" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="20.9" customWidth="1" min="7" max="7"/>
-    <col width="25.1" customWidth="1" min="8" max="8"/>
-    <col width="20.9" customWidth="1" min="9" max="9"/>
-    <col width="18.8" customWidth="1" min="10" max="10"/>
+    <col min="1" max="1" customWidth="true" width="2.5"/>
+    <col min="2" max="2" customWidth="true" width="23.0"/>
+    <col min="3" max="3" customWidth="true" width="70.0"/>
+    <col min="4" max="4" customWidth="true" width="15.7"/>
+    <col min="5" max="5" customWidth="true" width="23.0"/>
+    <col min="6" max="6" customWidth="true" width="23.0"/>
+    <col min="7" max="7" customWidth="true" width="20.9"/>
+    <col min="8" max="8" customWidth="true" width="25.1"/>
+    <col min="9" max="9" customWidth="true" width="20.9"/>
+    <col min="10" max="10" customWidth="true" width="18.8"/>
   </cols>
   <sheetData>
     <row r="2">

</xml_diff>